<commit_message>
feat: support company-specific config generation
</commit_message>
<xml_diff>
--- a/excel/sample-company.xlsx
+++ b/excel/sample-company.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fltnn\Documents\Codex\2026-07-04\concur-bot-web-sap-concur-1\outputs\concur-maigo-boshi-bot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DDB5929-04D4-46AB-AAFF-D103E4CF17AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44B556A0-338A-43BF-85F6-1675301B96BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="2" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" firstSheet="1" activeTab="2" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
   </bookViews>
   <sheets>
     <sheet name="01_基本設定" sheetId="8" r:id="rId1"/>
@@ -1479,7 +1479,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{124A85F1-4193-4290-83B0-CB7B0A187FD5}" name="テーブル68" displayName="テーブル68" ref="A1:D4" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{124A85F1-4193-4290-83B0-CB7B0A187FD5}" name="テーブル68" displayName="テーブル68" ref="A1:D4" totalsRowShown="0" headerRowDxfId="7">
   <autoFilter ref="A1:D4" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{A143BD03-D6FC-4045-A9B5-7AEDBC91E374}" name="会社ID"/>
@@ -1492,7 +1492,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{2AE807E6-FFF0-4D48-A8D6-3CA19EA411C3}" name="テーブル689" displayName="テーブル689" ref="A1:E4" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{2AE807E6-FFF0-4D48-A8D6-3CA19EA411C3}" name="テーブル689" displayName="テーブル689" ref="A1:E4" totalsRowShown="0" headerRowDxfId="6">
   <autoFilter ref="A1:E4" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{765DB1FB-9792-4378-B48E-9FB49A4A097F}" name="経費タイプ"/>
@@ -1506,7 +1506,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F4" totalsRowShown="0" headerRowDxfId="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F4" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="A1:F4" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{A203C0B4-DA8B-47FB-AD93-06B65D3DF83A}" name="申請内容"/>
@@ -1521,7 +1521,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D2" totalsRowShown="0" headerRowDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D2" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:D2" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{AB2A4918-1B3A-444C-8397-B8D718A1DCC8}" name="company_id"/>
@@ -1534,7 +1534,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}" name="テーブル2" displayName="テーブル2" ref="A1:D3" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}" name="テーブル2" displayName="テーブル2" ref="A1:D3" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="A1:D3" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{08666AA1-F4F1-499A-81C6-0435DF1C9F71}" name="policy_id"/>
@@ -1547,7 +1547,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}" name="テーブル3" displayName="テーブル3" ref="A1:E4" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}" name="テーブル3" displayName="テーブル3" ref="A1:E4" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:E4" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{DFC75CD8-2F06-42D1-80B3-9FF4CB20C500}" name="expense_type_id"/>
@@ -1561,7 +1561,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}" name="テーブル4" displayName="テーブル4" ref="A1:D4" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}" name="テーブル4" displayName="テーブル4" ref="A1:D4" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:D4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{49FF6D61-A7D7-4218-AFCD-AE85CAFCC4CE}" name="question_id"/>
@@ -1574,7 +1574,7 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}" name="テーブル5" displayName="テーブル5" ref="A1:D8" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}" name="テーブル5" displayName="テーブル5" ref="A1:D8" totalsRowShown="0" headerRowDxfId="1">
   <autoFilter ref="A1:D8" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{3682239B-A68F-4370-9ACB-BF52DFBFAD96}" name="question_id"/>
@@ -1587,7 +1587,7 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}" name="テーブル6" displayName="テーブル6" ref="A1:G8" totalsRowShown="0" headerRowDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}" name="テーブル6" displayName="テーブル6" ref="A1:G8" totalsRowShown="0" headerRowDxfId="0">
   <autoFilter ref="A1:G8" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{19828411-B567-413C-951E-9FC2EF9245C2}" name="rule_id"/>
@@ -2036,6 +2036,11 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576 D2:D1048576" xr:uid="{3B8B1928-C706-4E6C-86BC-A09C64FCA300}">
+      <formula1>"Y,N"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -2128,6 +2133,11 @@
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{8D3BCA68-F94E-4521-A386-BDAD8C1959B9}">
+      <formula1>"はい"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>

<commit_message>
feat: validate expense type settings
</commit_message>
<xml_diff>
--- a/excel/sample-company.xlsx
+++ b/excel/sample-company.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fltnn\Documents\Codex\2026-07-04\concur-bot-web-sap-concur-1\outputs\concur-maigo-boshi-bot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44B556A0-338A-43BF-85F6-1675301B96BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859A7200-8AC0-46A7-A312-33262AF343C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" firstSheet="1" activeTab="2" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
   </bookViews>
@@ -526,7 +526,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="85">
   <si>
     <t>company_id</t>
   </si>
@@ -782,6 +782,10 @@
   </si>
   <si>
     <t>出張時のみ</t>
+  </si>
+  <si>
+    <t>タクシー</t>
+    <phoneticPr fontId="1"/>
   </si>
 </sst>
 </file>
@@ -2102,10 +2106,10 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>24</v>
+        <v>84</v>
       </c>
       <c r="E3" t="s">
         <v>43</v>

</xml_diff>

<commit_message>
feat: add additional excel validators
</commit_message>
<xml_diff>
--- a/excel/sample-company.xlsx
+++ b/excel/sample-company.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fltnn\Documents\Codex\2026-07-04\concur-bot-web-sap-concur-1\outputs\concur-maigo-boshi-bot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{859A7200-8AC0-46A7-A312-33262AF343C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FD741C-B224-4AD8-B1AA-B5641D68E6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" firstSheet="1" activeTab="2" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
   </bookViews>
   <sheets>
     <sheet name="01_基本設定" sheetId="8" r:id="rId1"/>
@@ -526,7 +526,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="87">
   <si>
     <t>company_id</t>
   </si>
@@ -785,6 +785,17 @@
   </si>
   <si>
     <t>タクシー</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>normal_expense</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>サンプル会社</t>
+    <rPh sb="4" eb="6">
+      <t>カイシャ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -1510,7 +1521,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F4" totalsRowShown="0" headerRowDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F4" totalsRowShown="0" headerRowDxfId="5">
   <autoFilter ref="A1:F4" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{A203C0B4-DA8B-47FB-AD93-06B65D3DF83A}" name="申請内容"/>
@@ -1525,7 +1536,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D2" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D2" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="A1:D2" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{AB2A4918-1B3A-444C-8397-B8D718A1DCC8}" name="company_id"/>
@@ -2182,7 +2193,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>86</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -2333,7 +2344,7 @@
         <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>85</v>
       </c>
       <c r="C3" t="s">
         <v>24</v>
@@ -2350,7 +2361,7 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
         <v>63</v>
@@ -2365,7 +2376,7 @@
   </sheetData>
   <phoneticPr fontId="1"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576 E2:E1048576" xr:uid="{E9925988-1936-4F72-BF2A-86C37C8061C2}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:E1048576" xr:uid="{E9925988-1936-4F72-BF2A-86C37C8061C2}">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
refactor: improve validation error messages
</commit_message>
<xml_diff>
--- a/excel/sample-company.xlsx
+++ b/excel/sample-company.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fltnn\Documents\Codex\2026-07-04\concur-bot-web-sap-concur-1\outputs\concur-maigo-boshi-bot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05FD741C-B224-4AD8-B1AA-B5641D68E6E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE53F500-CE7B-4E2D-89DD-AED459039ECE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="3" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
   </bookViews>
   <sheets>
     <sheet name="01_基本設定" sheetId="8" r:id="rId1"/>
@@ -526,7 +526,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="88">
   <si>
     <t>company_id</t>
   </si>
@@ -792,10 +792,14 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>宿泊費</t>
+    <rPh sb="0" eb="3">
+      <t>シュクハクヒ</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
     <t>サンプル会社</t>
-    <rPh sb="4" eb="6">
-      <t>カイシャ</t>
-    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -2137,7 +2141,7 @@
         <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="E4" t="s">
         <v>65</v>
@@ -2193,7 +2197,7 @@
         <v>4</v>
       </c>
       <c r="B2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C2" t="s">
         <v>6</v>
@@ -2327,7 +2331,7 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
feat: use Excel metadata for required validation#
</commit_message>
<xml_diff>
--- a/excel/sample-company.xlsx
+++ b/excel/sample-company.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fltnn\Documents\Codex\2026-07-04\concur-bot-web-sap-concur-1\outputs\concur-maigo-boshi-bot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{733DE5E7-4688-444D-94E1-9376719CBE43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BE7108-B73D-4A72-8D5D-E01B6BA649A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="2" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
   </bookViews>
   <sheets>
     <sheet name="01_基本設定" sheetId="8" r:id="rId1"/>
@@ -789,13 +789,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>宿泊費</t>
-    <rPh sb="0" eb="3">
-      <t>シュクハクヒ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>サンプル会社</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -815,6 +808,13 @@
   </si>
   <si>
     <t>expense_type_id</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>宿泊費</t>
+    <rPh sb="0" eb="3">
+      <t>シュクハクヒ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -902,26 +902,23 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2196,7 +2193,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="10.4375" bestFit="1" customWidth="1"/>
@@ -2228,83 +2225,71 @@
     </row>
     <row r="2" spans="1:6" s="1" customFormat="1">
       <c r="A2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>88</v>
-      </c>
       <c r="C2" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>88</v>
-      </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="4" t="s">
+      <c r="A3" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4" t="s">
+      <c r="D3" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="4" t="s">
+      <c r="A4" t="s">
         <v>83</v>
       </c>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4" t="s">
+      <c r="D4" t="s">
         <v>83</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="F4" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="4" t="s">
+      <c r="A5" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" t="s">
         <v>47</v>
       </c>
-      <c r="C5" s="4"/>
-      <c r="D5" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="E5" s="4" t="s">
+      <c r="D5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E5" t="s">
         <v>64</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="4"/>
-      <c r="B6" s="4"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -2325,7 +2310,7 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="15.6875" bestFit="1" customWidth="1"/>
@@ -2349,38 +2334,32 @@
       </c>
     </row>
     <row r="2" spans="1:4" s="1" customFormat="1">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>88</v>
-      </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="4" t="s">
+      <c r="A3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="C3" s="4" t="s">
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="4"/>
-      <c r="B4" s="4"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1"/>
@@ -2428,43 +2407,43 @@
     </row>
     <row r="2" spans="1:4" s="1" customFormat="1">
       <c r="A2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>88</v>
-      </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="4" t="s">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="4" t="s">
+      <c r="A4" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="4">
+      <c r="D4">
         <v>2</v>
       </c>
     </row>
@@ -2501,7 +2480,7 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1">
       <c r="A1" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>8</v>
@@ -2518,69 +2497,69 @@
     </row>
     <row r="2" spans="1:5" s="1" customFormat="1">
       <c r="A2" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" s="4" t="s">
+      <c r="A3" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" s="4" t="s">
+      <c r="A4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>84</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" s="4" t="s">
+      <c r="A5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" t="s">
         <v>84</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: restore sample company Excel template style
</commit_message>
<xml_diff>
--- a/excel/sample-company.xlsx
+++ b/excel/sample-company.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fltnn\Documents\Codex\2026-07-04\concur-bot-web-sap-concur-1\outputs\concur-maigo-boshi-bot\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BE7108-B73D-4A72-8D5D-E01B6BA649A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3D70D819-6FDF-4B33-A933-68DAC6761E6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" activeTab="2" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="15675" firstSheet="1" activeTab="7" xr2:uid="{249C455E-F0B5-406B-89F2-4DE90A0306D5}"/>
   </bookViews>
   <sheets>
     <sheet name="01_基本設定" sheetId="8" r:id="rId1"/>
@@ -526,7 +526,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="122">
   <si>
     <t>company_id</t>
   </si>
@@ -717,38 +717,34 @@
     <t>領収書が不要な場合でも会社規定に従ってください。</t>
   </si>
   <si>
+    <t>r003</t>
+  </si>
+  <si>
+    <t>宿泊費を選択してください。</t>
+  </si>
+  <si>
+    <t>領収書添付が必要です。</t>
+  </si>
+  <si>
+    <t>申請内容</t>
+  </si>
+  <si>
+    <t>出張に関係</t>
+  </si>
+  <si>
+    <t>領収書あり</t>
+  </si>
+  <si>
+    <t>経費タイプ</t>
+  </si>
+  <si>
+    <t>案内メッセージ</t>
+  </si>
+  <si>
+    <t>注意事項</t>
+  </si>
+  <si>
     <t>宿泊費</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>r003</t>
-  </si>
-  <si>
-    <t>宿泊費を選択してください。</t>
-  </si>
-  <si>
-    <t>領収書添付が必要です。</t>
-  </si>
-  <si>
-    <t>申請内容</t>
-  </si>
-  <si>
-    <t>出張に関係</t>
-  </si>
-  <si>
-    <t>領収書あり</t>
-  </si>
-  <si>
-    <t>経費タイプ</t>
-  </si>
-  <si>
-    <t>案内メッセージ</t>
-  </si>
-  <si>
-    <t>注意事項</t>
-  </si>
-  <si>
-    <t>宿泊費</t>
   </si>
   <si>
     <t>会社ID</t>
@@ -779,14 +775,6 @@
   </si>
   <si>
     <t>出張時のみ</t>
-  </si>
-  <si>
-    <t>タクシー</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>normal_expense</t>
-    <phoneticPr fontId="1"/>
   </si>
   <si>
     <t>サンプル会社</t>
@@ -807,22 +795,122 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
+    <t>必須</t>
+  </si>
+  <si>
+    <t>任意</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>会食</t>
+  </si>
+  <si>
+    <t>会食費</t>
+  </si>
+  <si>
+    <t>会食は「会食費」を選択してください。</t>
+  </si>
+  <si>
+    <t>領収書を添付し、参加者・目的を記載してください。</t>
+  </si>
+  <si>
+    <t>接待</t>
+  </si>
+  <si>
+    <t>接待交際費</t>
+  </si>
+  <si>
+    <t>接待は「接待交際費」を選択してください。</t>
+  </si>
+  <si>
+    <t>取引先名・参加者・目的を記載してください。</t>
+  </si>
+  <si>
+    <t>備品購入</t>
+  </si>
+  <si>
+    <t>備品購入は「備品購入」を選択してください。</t>
+  </si>
+  <si>
+    <t>購入品名と業務利用目的を記載してください。</t>
+  </si>
+  <si>
+    <t>研修</t>
+  </si>
+  <si>
+    <t>研修費</t>
+  </si>
+  <si>
+    <t>研修・セミナーは「研修費」を選択してください。</t>
+  </si>
+  <si>
+    <t>研修名・受講日・業務関連性を記載してください。</t>
+  </si>
+  <si>
+    <t>通信費</t>
+  </si>
+  <si>
+    <t>通信費は「通信費」を選択してください。</t>
+  </si>
+  <si>
+    <t>月額利用料やオンラインサービス利用料の場合に利用します。</t>
+  </si>
+  <si>
+    <t>社内外の会議・会食で利用します。</t>
+  </si>
+  <si>
+    <t>取引先接待の場合に利用します。</t>
+  </si>
+  <si>
+    <t>業務利用の備品・消耗品購入で利用します。</t>
+  </si>
+  <si>
+    <t>業務研修・セミナー参加費で利用します。</t>
+  </si>
+  <si>
+    <t>通信料・オンラインサービス利用料で利用します。</t>
+  </si>
+  <si>
     <t>expense_type_id</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
-    <t>宿泊費</t>
-    <rPh sb="0" eb="3">
-      <t>シュクハクヒ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>dining</t>
+  </si>
+  <si>
+    <t>entertainment</t>
+  </si>
+  <si>
+    <t>equipment</t>
+  </si>
+  <si>
+    <t>training</t>
+  </si>
+  <si>
+    <t>communication</t>
+  </si>
+  <si>
+    <t>r004</t>
+  </si>
+  <si>
+    <t>r005</t>
+  </si>
+  <si>
+    <t>r006</t>
+  </si>
+  <si>
+    <t>r007</t>
+  </si>
+  <si>
+    <t>r008</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -873,6 +961,21 @@
       <charset val="128"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="游ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -902,7 +1005,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -921,28 +1024,40 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="9">
+  <dxfs count="28">
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
       </font>
     </dxf>
     <dxf>
@@ -957,12 +1072,18 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color theme="0"/>
         <name val="游ゴシック"/>
         <family val="3"/>
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -976,12 +1097,18 @@
         <u val="none"/>
         <vertAlign val="baseline"/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color theme="0"/>
         <name val="游ゴシック"/>
         <family val="3"/>
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <font>
@@ -1112,44 +1239,6 @@
         <charset val="128"/>
         <scheme val="minor"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="游ゴシック"/>
-        <family val="3"/>
-        <charset val="128"/>
-        <scheme val="minor"/>
-      </font>
       <border diagonalUp="0" diagonalDown="0">
         <left style="thin">
           <color indexed="64"/>
@@ -1166,6 +1255,151 @@
           <color indexed="64"/>
         </horizontal>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="游ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="8" tint="-0.249977111117893"/>
+        </patternFill>
+      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1619,7 +1853,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{124A85F1-4193-4290-83B0-CB7B0A187FD5}" name="テーブル68" displayName="テーブル68" ref="A1:D4" totalsRowShown="0" headerRowDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{124A85F1-4193-4290-83B0-CB7B0A187FD5}" name="テーブル68" displayName="テーブル68" ref="A1:D4" totalsRowShown="0" headerRowDxfId="18">
   <autoFilter ref="A1:D4" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{A143BD03-D6FC-4045-A9B5-7AEDBC91E374}" name="会社ID"/>
@@ -1627,27 +1861,27 @@
     <tableColumn id="3" xr3:uid="{9F770A3E-49C8-4946-96D2-777EB3CF2E3D}" name="デフォルトポリシー"/>
     <tableColumn id="4" xr3:uid="{AF941CDE-F1CF-4EEC-AF8B-C8A3A9ACC4C1}" name="言語"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{2AE807E6-FFF0-4D48-A8D6-3CA19EA411C3}" name="テーブル689" displayName="テーブル689" ref="A1:E4" totalsRowShown="0" headerRowDxfId="6">
-  <autoFilter ref="A1:E4" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{2AE807E6-FFF0-4D48-A8D6-3CA19EA411C3}" name="テーブル689" displayName="テーブル689" ref="A1:E9" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+  <autoFilter ref="A1:E9" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{765DB1FB-9792-4378-B48E-9FB49A4A097F}" name="経費タイプ"/>
-    <tableColumn id="2" xr3:uid="{A3AC0354-9967-4FAA-A75A-034D4B6C345F}" name="ポリシー"/>
-    <tableColumn id="3" xr3:uid="{F98BB76D-0186-45A3-AD70-D0454600EF9F}" name="領収書要否"/>
-    <tableColumn id="4" xr3:uid="{8B0404ED-44A8-4358-8ACC-5B3F77A8D859}" name="使用有無"/>
-    <tableColumn id="5" xr3:uid="{1BD92D55-2C43-4EE6-89FE-A801B54928F4}" name="注意事項"/>
+    <tableColumn id="1" xr3:uid="{765DB1FB-9792-4378-B48E-9FB49A4A097F}" name="経費タイプ" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{A3AC0354-9967-4FAA-A75A-034D4B6C345F}" name="ポリシー" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{F98BB76D-0186-45A3-AD70-D0454600EF9F}" name="領収書要否" dataDxfId="13"/>
+    <tableColumn id="4" xr3:uid="{8B0404ED-44A8-4358-8ACC-5B3F77A8D859}" name="使用有無" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{1BD92D55-2C43-4EE6-89FE-A801B54928F4}" name="注意事項" dataDxfId="11"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F5" totalsRowShown="0" headerRowDxfId="8">
-  <autoFilter ref="A1:F5" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F10" totalsRowShown="0" headerRowDxfId="10">
+  <autoFilter ref="A1:F10" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{A203C0B4-DA8B-47FB-AD93-06B65D3DF83A}" name="申請内容"/>
     <tableColumn id="2" xr3:uid="{0FA34334-E5B3-4C7F-AAB6-BB1D856C1D66}" name="出張に関係"/>
@@ -1661,7 +1895,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D3" totalsRowShown="0" headerRowDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D3" totalsRowShown="0" headerRowDxfId="9">
   <autoFilter ref="A1:D3" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{AB2A4918-1B3A-444C-8397-B8D718A1DCC8}" name="company_id"/>
@@ -1674,7 +1908,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}" name="テーブル2" displayName="テーブル2" ref="A1:D4" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}" name="テーブル2" displayName="テーブル2" ref="A1:D4" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="A1:D4" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{08666AA1-F4F1-499A-81C6-0435DF1C9F71}" name="policy_id"/>
@@ -1687,8 +1921,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}" name="テーブル3" displayName="テーブル3" ref="A1:E5" totalsRowShown="0" headerRowDxfId="3">
-  <autoFilter ref="A1:E5" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}" name="テーブル3" displayName="テーブル3" ref="A1:E10" totalsRowShown="0" headerRowDxfId="7">
+  <autoFilter ref="A1:E10" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{DFC75CD8-2F06-42D1-80B3-9FF4CB20C500}" name="expense_type_id"/>
     <tableColumn id="2" xr3:uid="{324312A7-D2F2-4928-A9AB-3A204186A333}" name="policy_id"/>
@@ -1701,7 +1935,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}" name="テーブル4" displayName="テーブル4" ref="A1:D4" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}" name="テーブル4" displayName="テーブル4" ref="A1:D4" totalsRowShown="0" headerRowDxfId="6">
   <autoFilter ref="A1:D4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{49FF6D61-A7D7-4218-AFCD-AE85CAFCC4CE}" name="question_id"/>
@@ -1709,36 +1943,36 @@
     <tableColumn id="3" xr3:uid="{267E2B78-3308-417F-A46B-57905CC8F86C}" name="question_type"/>
     <tableColumn id="4" xr3:uid="{CF009CF6-40A0-451E-9B18-49C260EC4576}" name="display_order"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}" name="テーブル5" displayName="テーブル5" ref="A1:D8" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:D8" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}" name="テーブル5" displayName="テーブル5" ref="A1:D13" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+  <autoFilter ref="A1:D13" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{3682239B-A68F-4370-9ACB-BF52DFBFAD96}" name="question_id"/>
-    <tableColumn id="2" xr3:uid="{CB33AE30-AB6D-4B42-8EA6-F18C47A75D23}" name="option_label"/>
-    <tableColumn id="3" xr3:uid="{1CF0CE5F-7F1B-45ED-B75D-AF38ED3DADAA}" name="option_value"/>
-    <tableColumn id="4" xr3:uid="{20B66DDF-2E63-47EA-98AB-C8B52ED94200}" name="next_question_id"/>
+    <tableColumn id="1" xr3:uid="{3682239B-A68F-4370-9ACB-BF52DFBFAD96}" name="question_id" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{CB33AE30-AB6D-4B42-8EA6-F18C47A75D23}" name="option_label" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{1CF0CE5F-7F1B-45ED-B75D-AF38ED3DADAA}" name="option_value" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{20B66DDF-2E63-47EA-98AB-C8B52ED94200}" name="next_question_id" dataDxfId="0"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}" name="テーブル6" displayName="テーブル6" ref="A1:G8" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:G8" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}" name="テーブル6" displayName="テーブル6" ref="A1:G15" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+  <autoFilter ref="A1:G15" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{19828411-B567-413C-951E-9FC2EF9245C2}" name="rule_id"/>
-    <tableColumn id="2" xr3:uid="{3625B637-0E8B-479C-A351-334F9E08C7B1}" name="priority"/>
-    <tableColumn id="3" xr3:uid="{F62F4A9E-3FB0-4784-AB89-F7443CEB66CC}" name="condition_key"/>
-    <tableColumn id="4" xr3:uid="{E31981C1-F11F-4BC0-A905-EFFFFD9E06CE}" name="condition_value"/>
-    <tableColumn id="5" xr3:uid="{CB630B8B-2506-4CBD-92F1-EAAF054DB046}" name="result_expense_type_id"/>
-    <tableColumn id="6" xr3:uid="{BC06978D-C5E1-40A5-9214-793F4807C77B}" name="guidance_message"/>
-    <tableColumn id="7" xr3:uid="{3C1BFA58-FF4D-444E-8B3E-500A6063C815}" name="warning_message"/>
+    <tableColumn id="1" xr3:uid="{19828411-B567-413C-951E-9FC2EF9245C2}" name="rule_id" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{3625B637-0E8B-479C-A351-334F9E08C7B1}" name="priority" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{F62F4A9E-3FB0-4784-AB89-F7443CEB66CC}" name="condition_key" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{E31981C1-F11F-4BC0-A905-EFFFFD9E06CE}" name="condition_value" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{CB630B8B-2506-4CBD-92F1-EAAF054DB046}" name="result_expense_type_id" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{BC06978D-C5E1-40A5-9214-793F4807C77B}" name="guidance_message" dataDxfId="20"/>
+    <tableColumn id="7" xr3:uid="{3C1BFA58-FF4D-444E-8B3E-500A6063C815}" name="warning_message" dataDxfId="19"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -2054,17 +2288,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -2095,83 +2329,168 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="15.8125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.4375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.9375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="51.9375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="1" t="s">
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="6" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="1:5">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="B4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D9" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
-      <c r="A3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
-      <c r="A4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s">
-        <v>82</v>
+      <c r="E9" s="6" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -2193,7 +2512,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="10.4375" bestFit="1" customWidth="1"/>
@@ -2203,92 +2522,204 @@
     <col min="6" max="6" width="51.9375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="1" customFormat="1">
+    <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="F1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" s="1" customFormat="1">
-      <c r="A2" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" s="3" t="s">
+      <c r="E5" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C6" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="C7" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="C8" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E3" t="s">
-        <v>40</v>
-      </c>
-      <c r="F3" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>83</v>
-      </c>
-      <c r="D4" t="s">
-        <v>83</v>
-      </c>
-      <c r="E4" t="s">
-        <v>42</v>
-      </c>
-      <c r="F4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="D8" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="D5" t="s">
-        <v>89</v>
-      </c>
-      <c r="E5" t="s">
-        <v>64</v>
-      </c>
-      <c r="F5" t="s">
-        <v>65</v>
+      <c r="D9" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2335,16 +2766,16 @@
     </row>
     <row r="2" spans="1:4" s="1" customFormat="1">
       <c r="A2" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2352,7 +2783,7 @@
         <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -2407,16 +2838,16 @@
     </row>
     <row r="2" spans="1:4" s="1" customFormat="1">
       <c r="A2" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2468,7 +2899,7 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="17.0625" customWidth="1"/>
@@ -2478,9 +2909,9 @@
     <col min="5" max="5" width="7.6875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="1" customFormat="1">
+    <row r="1" spans="1:5">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>111</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>8</v>
@@ -2495,71 +2926,156 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:5" s="1" customFormat="1">
+    <row r="2" spans="1:5">
       <c r="A2" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:5">
-      <c r="A3" t="s">
+      <c r="A3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B3" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:5">
-      <c r="A4" t="s">
+      <c r="A4" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C4" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:5">
-      <c r="A5" t="s">
+      <c r="A5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="B5" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="E10" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2594,16 +3110,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -2670,110 +3186,192 @@
   <sheetPr>
     <tabColor rgb="FF00B050"/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="5" width="28.4375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" t="s">
+      <c r="A3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" t="s">
+      <c r="A4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" t="s">
+      <c r="A5" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="6" t="s">
         <v>48</v>
       </c>
+      <c r="D5" s="6" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="6" spans="1:4">
-      <c r="A6" t="s">
+      <c r="A6" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="6" t="s">
         <v>50</v>
       </c>
+      <c r="D6" s="6" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="7" spans="1:4">
-      <c r="A7" t="s">
+      <c r="A7" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="6" t="s">
         <v>48</v>
       </c>
+      <c r="D7" s="6" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="8" spans="1:4">
-      <c r="A8" t="s">
+      <c r="A8" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="6" t="s">
         <v>50</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -2792,7 +3390,7 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultRowHeight="17.649999999999999"/>
   <cols>
     <col min="1" max="1" width="8.375" customWidth="1"/>
@@ -2806,142 +3404,349 @@
     <col min="9" max="9" width="51.9375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:7">
+      <c r="A1" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" t="s">
+      <c r="A2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="6">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:7">
-      <c r="A3" t="s">
+      <c r="A3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="6">
         <v>1</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" t="s">
+      <c r="A4" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="6" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" t="s">
+      <c r="A5" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="6">
+        <v>3</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B5">
+      <c r="G5" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" s="6">
         <v>3</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B7" s="6">
+        <v>4</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E5" t="s">
-        <v>24</v>
-      </c>
-      <c r="F5" t="s">
-        <v>64</v>
-      </c>
-      <c r="G5" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="D7" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B8" s="6">
+        <v>4</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F6" t="s">
-        <v>64</v>
-      </c>
-      <c r="G6" t="s">
-        <v>65</v>
+      <c r="E8" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" s="6">
+        <v>5</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B10" s="6">
+        <v>5</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B11" s="6">
+        <v>6</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B12" s="6">
+        <v>6</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B13" s="6">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="B14" s="6">
+        <v>7</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="B15" s="6">
+        <v>8</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: skip Excel description rows when generating config
</commit_message>
<xml_diff>
--- a/excel/sample-company.xlsx
+++ b/excel/sample-company.xlsx
@@ -1062,6 +1062,21 @@
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
@@ -1335,21 +1350,6 @@
           <bgColor theme="8" tint="-0.249977111117893"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -1853,7 +1853,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{124A85F1-4193-4290-83B0-CB7B0A187FD5}" name="テーブル68" displayName="テーブル68" ref="A1:D4" totalsRowShown="0" headerRowDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{124A85F1-4193-4290-83B0-CB7B0A187FD5}" name="テーブル68" displayName="テーブル68" ref="A1:D4" totalsRowShown="0" headerRowDxfId="21">
   <autoFilter ref="A1:D4" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{A143BD03-D6FC-4045-A9B5-7AEDBC91E374}" name="会社ID"/>
@@ -1866,21 +1866,21 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{2AE807E6-FFF0-4D48-A8D6-3CA19EA411C3}" name="テーブル689" displayName="テーブル689" ref="A1:E9" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{2AE807E6-FFF0-4D48-A8D6-3CA19EA411C3}" name="テーブル689" displayName="テーブル689" ref="A1:E9" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="A1:E9" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{765DB1FB-9792-4378-B48E-9FB49A4A097F}" name="経費タイプ" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{A3AC0354-9967-4FAA-A75A-034D4B6C345F}" name="ポリシー" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{F98BB76D-0186-45A3-AD70-D0454600EF9F}" name="領収書要否" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{8B0404ED-44A8-4358-8ACC-5B3F77A8D859}" name="使用有無" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{1BD92D55-2C43-4EE6-89FE-A801B54928F4}" name="注意事項" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{765DB1FB-9792-4378-B48E-9FB49A4A097F}" name="経費タイプ" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{A3AC0354-9967-4FAA-A75A-034D4B6C345F}" name="ポリシー" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{F98BB76D-0186-45A3-AD70-D0454600EF9F}" name="領収書要否" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{8B0404ED-44A8-4358-8ACC-5B3F77A8D859}" name="使用有無" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{1BD92D55-2C43-4EE6-89FE-A801B54928F4}" name="注意事項" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F10" totalsRowShown="0" headerRowDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{D84F3076-8FA9-4A7A-B033-E1CE7B7151AB}" name="テーブル68910" displayName="テーブル68910" ref="A1:F10" totalsRowShown="0" headerRowDxfId="13">
   <autoFilter ref="A1:F10" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{A203C0B4-DA8B-47FB-AD93-06B65D3DF83A}" name="申請内容"/>
@@ -1895,7 +1895,7 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D3" totalsRowShown="0" headerRowDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}" name="テーブル1" displayName="テーブル1" ref="A1:D3" totalsRowShown="0" headerRowDxfId="12">
   <autoFilter ref="A1:D3" xr:uid="{1C076EDE-3A14-44A0-A174-6B7535F7CD49}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{AB2A4918-1B3A-444C-8397-B8D718A1DCC8}" name="company_id"/>
@@ -1908,7 +1908,7 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}" name="テーブル2" displayName="テーブル2" ref="A1:D4" totalsRowShown="0" headerRowDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}" name="テーブル2" displayName="テーブル2" ref="A1:D4" totalsRowShown="0" headerRowDxfId="11">
   <autoFilter ref="A1:D4" xr:uid="{B996CD8C-0A29-479E-8E8E-B660E8186F1E}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{08666AA1-F4F1-499A-81C6-0435DF1C9F71}" name="policy_id"/>
@@ -1921,7 +1921,7 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}" name="テーブル3" displayName="テーブル3" ref="A1:E10" totalsRowShown="0" headerRowDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}" name="テーブル3" displayName="テーブル3" ref="A1:E10" totalsRowShown="0" headerRowDxfId="10">
   <autoFilter ref="A1:E10" xr:uid="{39899102-F42A-45C7-B14D-05C2499F2811}"/>
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{DFC75CD8-2F06-42D1-80B3-9FF4CB20C500}" name="expense_type_id"/>
@@ -1935,7 +1935,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}" name="テーブル4" displayName="テーブル4" ref="A1:D4" totalsRowShown="0" headerRowDxfId="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}" name="テーブル4" displayName="テーブル4" ref="A1:D4" totalsRowShown="0" headerRowDxfId="9">
   <autoFilter ref="A1:D4" xr:uid="{0426B32E-8DD3-4337-B275-388375226821}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{49FF6D61-A7D7-4218-AFCD-AE85CAFCC4CE}" name="question_id"/>
@@ -1948,29 +1948,29 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}" name="テーブル5" displayName="テーブル5" ref="A1:D13" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}" name="テーブル5" displayName="テーブル5" ref="A1:D13" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
   <autoFilter ref="A1:D13" xr:uid="{A21320F6-ACAD-46FD-9E8A-75616BA2BCE7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{3682239B-A68F-4370-9ACB-BF52DFBFAD96}" name="question_id" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{CB33AE30-AB6D-4B42-8EA6-F18C47A75D23}" name="option_label" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{1CF0CE5F-7F1B-45ED-B75D-AF38ED3DADAA}" name="option_value" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{20B66DDF-2E63-47EA-98AB-C8B52ED94200}" name="next_question_id" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{3682239B-A68F-4370-9ACB-BF52DFBFAD96}" name="question_id" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{CB33AE30-AB6D-4B42-8EA6-F18C47A75D23}" name="option_label" dataDxfId="24"/>
+    <tableColumn id="3" xr3:uid="{1CF0CE5F-7F1B-45ED-B75D-AF38ED3DADAA}" name="option_value" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{20B66DDF-2E63-47EA-98AB-C8B52ED94200}" name="next_question_id" dataDxfId="22"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}" name="テーブル6" displayName="テーブル6" ref="A1:G15" totalsRowShown="0" headerRowDxfId="27" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}" name="テーブル6" displayName="テーブル6" ref="A1:G15" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
   <autoFilter ref="A1:G15" xr:uid="{54DCA0F0-87B2-47C2-9395-4E6E1CFBB1D6}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{19828411-B567-413C-951E-9FC2EF9245C2}" name="rule_id" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{3625B637-0E8B-479C-A351-334F9E08C7B1}" name="priority" dataDxfId="24"/>
-    <tableColumn id="3" xr3:uid="{F62F4A9E-3FB0-4784-AB89-F7443CEB66CC}" name="condition_key" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{E31981C1-F11F-4BC0-A905-EFFFFD9E06CE}" name="condition_value" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{CB630B8B-2506-4CBD-92F1-EAAF054DB046}" name="result_expense_type_id" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{BC06978D-C5E1-40A5-9214-793F4807C77B}" name="guidance_message" dataDxfId="20"/>
-    <tableColumn id="7" xr3:uid="{3C1BFA58-FF4D-444E-8B3E-500A6063C815}" name="warning_message" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{19828411-B567-413C-951E-9FC2EF9245C2}" name="rule_id" dataDxfId="6"/>
+    <tableColumn id="2" xr3:uid="{3625B637-0E8B-479C-A351-334F9E08C7B1}" name="priority" dataDxfId="5"/>
+    <tableColumn id="3" xr3:uid="{F62F4A9E-3FB0-4784-AB89-F7443CEB66CC}" name="condition_key" dataDxfId="4"/>
+    <tableColumn id="4" xr3:uid="{E31981C1-F11F-4BC0-A905-EFFFFD9E06CE}" name="condition_value" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{CB630B8B-2506-4CBD-92F1-EAAF054DB046}" name="result_expense_type_id" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{BC06978D-C5E1-40A5-9214-793F4807C77B}" name="guidance_message" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{3C1BFA58-FF4D-444E-8B3E-500A6063C815}" name="warning_message" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>